<commit_message>
file updates including masterdatabase
</commit_message>
<xml_diff>
--- a/data/code_book.xlsx
+++ b/data/code_book.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10512"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericfoerster/Desktop/torv-reports/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericfoerster/Desktop/torv-reports v4/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D23FD2F-0906-D241-ABFC-AADBE4DE600E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{962B51C3-640A-F947-A2AC-9D59FFF194BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18100" yWindow="500" windowWidth="22820" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22340" yWindow="500" windowWidth="22820" windowHeight="26600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="client_list" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1420" uniqueCount="1128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="1134">
   <si>
     <t>client_number</t>
   </si>
@@ -3411,6 +3411,24 @@
   </si>
   <si>
     <t>DOMINION</t>
+  </si>
+  <si>
+    <t>Adobe Creek National Golf Course</t>
+  </si>
+  <si>
+    <t>Chipeta Golf Course</t>
+  </si>
+  <si>
+    <t>S022</t>
+  </si>
+  <si>
+    <t>Organic Matter % at 440C and Sand Fractions</t>
+  </si>
+  <si>
+    <t>ADOBE</t>
+  </si>
+  <si>
+    <t>CHIPETA</t>
   </si>
 </sst>
 </file>
@@ -3980,9 +3998,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4020,7 +4038,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4126,7 +4144,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4268,7 +4286,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4276,7 +4294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -4569,6 +4587,22 @@
       </c>
       <c r="B36" t="s">
         <v>1126</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>92138</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1128</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>92128</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1129</v>
       </c>
     </row>
   </sheetData>
@@ -4586,7 +4620,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B614"/>
+  <dimension ref="A1:B615"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -9457,6 +9491,14 @@
       </c>
       <c r="B614" t="s">
         <v>1057</v>
+      </c>
+    </row>
+    <row r="615" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A615" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B615" t="s">
+        <v>1131</v>
       </c>
     </row>
   </sheetData>
@@ -9680,7 +9722,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8789E2A9-FDC3-4E71-8044-B16DA9DC3A5E}">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.6640625" bestFit="1" customWidth="1"/>
@@ -10150,6 +10192,28 @@
         <v>1072</v>
       </c>
     </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1072</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1072</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Report updates — templates, data, and Trail Creek client additions
Updated water, OM, trendline, and sand fraction templates. Revised
ai-report-prompt.md. Added Trail Creek to eric.R. Updated MASTER_DATABASE
and code book with latest data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/code_book.xlsx
+++ b/data/code_book.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericfoerster/Desktop/ torv-reports v4/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ACA2CC-2AD0-4E45-BDBF-F7A3FF661AD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85B19C74-C0D4-4D47-AAC8-700F3C51142E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16160" yWindow="600" windowWidth="35040" windowHeight="26060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1500" yWindow="600" windowWidth="35040" windowHeight="26060" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="client_list" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1507" uniqueCount="1174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="1178">
   <si>
     <t>client_number</t>
   </si>
@@ -3549,6 +3549,18 @@
   </si>
   <si>
     <t>HERITAGE</t>
+  </si>
+  <si>
+    <t>Sun Valley Resort White Clouds Golf Course</t>
+  </si>
+  <si>
+    <t>Sun Valley Resort Trail Creek Golf Course</t>
+  </si>
+  <si>
+    <t>WHITECLOUDS</t>
+  </si>
+  <si>
+    <t>TRAILCREEK</t>
   </si>
 </sst>
 </file>
@@ -4414,7 +4426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -4870,8 +4882,27 @@
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>96231</v>
+      </c>
       <c r="B57" t="s">
         <v>1172</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>96459</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>96461</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1175</v>
       </c>
     </row>
   </sheetData>
@@ -10000,7 +10031,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8789E2A9-FDC3-4E71-8044-B16DA9DC3A5E}">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="40.6640625" bestFit="1" customWidth="1"/>
@@ -10701,6 +10732,28 @@
         <v>1077</v>
       </c>
     </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>1174</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1071</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>